<commit_message>
Added standard templates and modified dimensions sheet
</commit_message>
<xml_diff>
--- a/cad/dimensions.xlsx
+++ b/cad/dimensions.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27928"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28025"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tallA\Repos\VolumanXR\hardware-capture\cad\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{267678F9-D9F0-4E15-B056-FE22A2BDEFEE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A91EABF6-0DFC-4CFA-9810-4A19FD76F306}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="25440" windowHeight="15390" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-10785" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="14">
   <si>
     <t>Parameter Name</t>
   </si>
@@ -37,6 +37,36 @@
   </si>
   <si>
     <t>Comment</t>
+  </si>
+  <si>
+    <t>d_tol</t>
+  </si>
+  <si>
+    <t>mm</t>
+  </si>
+  <si>
+    <t>d_wand</t>
+  </si>
+  <si>
+    <t>Wanddicke (Schalung)</t>
+  </si>
+  <si>
+    <t>Toleranzmaß 3D-Druck</t>
+  </si>
+  <si>
+    <t>m</t>
+  </si>
+  <si>
+    <t>Profillänge Kameratraeger</t>
+  </si>
+  <si>
+    <t>l_profil_traeger</t>
+  </si>
+  <si>
+    <t>l_profil_staender</t>
+  </si>
+  <si>
+    <t>Profillänge Staenderprofil</t>
   </si>
 </sst>
 </file>
@@ -354,7 +384,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D1"/>
+  <dimension ref="A1:D5"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="19.5703125" customWidth="1"/>
@@ -374,6 +404,62 @@
         <v>3</v>
       </c>
     </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>4</v>
+      </c>
+      <c r="B2">
+        <v>0.3</v>
+      </c>
+      <c r="C2" t="s">
+        <v>5</v>
+      </c>
+      <c r="D2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>6</v>
+      </c>
+      <c r="B3">
+        <v>1.5</v>
+      </c>
+      <c r="C3" t="s">
+        <v>5</v>
+      </c>
+      <c r="D3" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>11</v>
+      </c>
+      <c r="B4">
+        <v>1.5</v>
+      </c>
+      <c r="C4" t="s">
+        <v>9</v>
+      </c>
+      <c r="D4" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>12</v>
+      </c>
+      <c r="B5">
+        <v>2.5</v>
+      </c>
+      <c r="C5" t="s">
+        <v>9</v>
+      </c>
+      <c r="D5" t="s">
+        <v>13</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
finished cad construction of alu profiles for rig
</commit_message>
<xml_diff>
--- a/cad/dimensions.xlsx
+++ b/cad/dimensions.xlsx
@@ -8,24 +8,35 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tallA\Repos\VolumanXR\hardware-capture\cad\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A91EABF6-0DFC-4CFA-9810-4A19FD76F306}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6FBF32CE-13C0-4940-9FD2-8B4EBC454176}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-10785" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="22">
   <si>
     <t>Parameter Name</t>
   </si>
@@ -60,13 +71,37 @@
     <t>Profillänge Kameratraeger</t>
   </si>
   <si>
-    <t>l_profil_traeger</t>
-  </si>
-  <si>
-    <t>l_profil_staender</t>
-  </si>
-  <si>
     <t>Profillänge Staenderprofil</t>
+  </si>
+  <si>
+    <t>d_traeger</t>
+  </si>
+  <si>
+    <t>Abstand träger horizontal</t>
+  </si>
+  <si>
+    <t>l_profil_40x40</t>
+  </si>
+  <si>
+    <t>l_profil_20x20</t>
+  </si>
+  <si>
+    <t>b_profil_20x20</t>
+  </si>
+  <si>
+    <t>h_profil_20x20</t>
+  </si>
+  <si>
+    <t>b_profil_40x40</t>
+  </si>
+  <si>
+    <t>h_profil_40x40</t>
+  </si>
+  <si>
+    <t>D_oct</t>
+  </si>
+  <si>
+    <t>Durchmesser Oktagon (Distanz gegenüberliegende Seiten)</t>
   </si>
 </sst>
 </file>
@@ -384,7 +419,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D5"/>
+  <dimension ref="A1:D11"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="19.5703125" customWidth="1"/>
@@ -434,7 +469,7 @@
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="B4">
         <v>1.5</v>
@@ -448,7 +483,7 @@
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B5">
         <v>2.5</v>
@@ -457,7 +492,81 @@
         <v>9</v>
       </c>
       <c r="D5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>12</v>
+      </c>
+      <c r="B6">
+        <f>B5/4</f>
+        <v>0.625</v>
+      </c>
+      <c r="C6" t="s">
+        <v>9</v>
+      </c>
+      <c r="D6" t="s">
         <v>13</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>16</v>
+      </c>
+      <c r="B7">
+        <v>20</v>
+      </c>
+      <c r="C7" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>17</v>
+      </c>
+      <c r="B8">
+        <v>20</v>
+      </c>
+      <c r="C8" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>18</v>
+      </c>
+      <c r="B9">
+        <v>40</v>
+      </c>
+      <c r="C9" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>19</v>
+      </c>
+      <c r="B10">
+        <v>40</v>
+      </c>
+      <c r="C10" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>20</v>
+      </c>
+      <c r="B11">
+        <f>(B4*10^3-2*B7/2)*(1+SQRT(2))</f>
+        <v>3573.0360723121803</v>
+      </c>
+      <c r="C11" t="s">
+        <v>5</v>
+      </c>
+      <c r="D11" t="s">
+        <v>21</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Reworked rig into rig_v2
Connections betweens aluminium profiles is now realised with lasercut 45deg connectors
</commit_message>
<xml_diff>
--- a/cad/dimensions.xlsx
+++ b/cad/dimensions.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tallA\Repos\VolumanXR\hardware-capture\cad\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6FBF32CE-13C0-4940-9FD2-8B4EBC454176}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{183F7AA0-0FFC-45D4-80B7-8249ECE32A2A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-10785" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-15630" windowWidth="19440" windowHeight="15000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -559,8 +559,8 @@
         <v>20</v>
       </c>
       <c r="B11">
-        <f>(B4*10^3-2*B7/2)*(1+SQRT(2))</f>
-        <v>3573.0360723121803</v>
+        <f>(B4*10^3)*(1+SQRT(2))</f>
+        <v>3621.3203435596424</v>
       </c>
       <c r="C11" t="s">
         <v>5</v>

</xml_diff>

<commit_message>
Added camera holder (WIP)
</commit_message>
<xml_diff>
--- a/cad/dimensions.xlsx
+++ b/cad/dimensions.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tallA\Repos\VolumanXR\hardware-capture\cad\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ABBB0CA3-E3B1-4523-8C39-BD899870703B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FA790DE2-71A4-4120-B0C6-4F75E249DC14}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2835" yWindow="2730" windowWidth="18900" windowHeight="11055" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-26070" yWindow="-5220" windowWidth="18900" windowHeight="11055" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="30">
   <si>
     <t>Parameter Name</t>
   </si>
@@ -108,6 +108,24 @@
   </si>
   <si>
     <t>D_hexadeca</t>
+  </si>
+  <si>
+    <t>l_rasp_pi</t>
+  </si>
+  <si>
+    <t>Länge Raspberry Pi</t>
+  </si>
+  <si>
+    <t>b_rasp_pi</t>
+  </si>
+  <si>
+    <t>Breite Raspberry Pi</t>
+  </si>
+  <si>
+    <t>r_rasp_pi</t>
+  </si>
+  <si>
+    <t>Rundung Raspberry Pi</t>
   </si>
 </sst>
 </file>
@@ -425,7 +443,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D12"/>
+  <dimension ref="A1:D15"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="19.5703125" customWidth="1"/>
@@ -591,6 +609,48 @@
         <v>22</v>
       </c>
     </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>24</v>
+      </c>
+      <c r="B13">
+        <v>85</v>
+      </c>
+      <c r="C13" t="s">
+        <v>5</v>
+      </c>
+      <c r="D13" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>26</v>
+      </c>
+      <c r="B14">
+        <v>56</v>
+      </c>
+      <c r="C14" t="s">
+        <v>5</v>
+      </c>
+      <c r="D14" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>28</v>
+      </c>
+      <c r="B15">
+        <v>3</v>
+      </c>
+      <c r="C15" t="s">
+        <v>5</v>
+      </c>
+      <c r="D15" t="s">
+        <v>29</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Revised Cameraholder of top row
Adjusted according to the vertical viewing angle to angle the cameras downwards for better coverage
</commit_message>
<xml_diff>
--- a/cad/dimensions.xlsx
+++ b/cad/dimensions.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28025"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28129"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tallA\Repos\VolumanXR\hardware-capture\cad\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FA790DE2-71A4-4120-B0C6-4F75E249DC14}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{17F87369-460A-4CD4-9F50-4E1DBF1316FD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-26070" yWindow="-5220" windowWidth="18900" windowHeight="11055" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-10785" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="35">
   <si>
     <t>Parameter Name</t>
   </si>
@@ -126,6 +126,21 @@
   </si>
   <si>
     <t>Rundung Raspberry Pi</t>
+  </si>
+  <si>
+    <t>w_kamera_hori</t>
+  </si>
+  <si>
+    <t>deg</t>
+  </si>
+  <si>
+    <t>Horizontaler Öffnungswinkel</t>
+  </si>
+  <si>
+    <t>w_kamera_vert</t>
+  </si>
+  <si>
+    <t>Vertikaler Öffnungswinkel</t>
   </si>
 </sst>
 </file>
@@ -443,7 +458,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D15"/>
+  <dimension ref="A1:D17"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="19.5703125" customWidth="1"/>
@@ -651,6 +666,34 @@
         <v>29</v>
       </c>
     </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>30</v>
+      </c>
+      <c r="B16">
+        <v>66</v>
+      </c>
+      <c r="C16" t="s">
+        <v>31</v>
+      </c>
+      <c r="D16" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>33</v>
+      </c>
+      <c r="B17">
+        <v>41</v>
+      </c>
+      <c r="C17" t="s">
+        <v>31</v>
+      </c>
+      <c r="D17" t="s">
+        <v>34</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>